<commit_message>
refine dashboard copy and demo student names
</commit_message>
<xml_diff>
--- a/outputs/teacher_support_studio/teacher_support_name_mapping.xlsx
+++ b/outputs/teacher_support_studio/teacher_support_name_mapping.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R1c8955ff6411475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="2" r:id="R04faef7b08874dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="3" r:id="Re5fb2ea508b04e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rd0969abef33b48ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="2" r:id="R20d65c7189cf4962"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="3" r:id="Rb9aed3051f5b4853"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -622,7 +622,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f65d0d7dbdc446d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54530cd7643d4d00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -667,7 +667,7 @@
         <x:v>64634</x:v>
       </x:c>
       <x:c r="C2" s="16" t="str">
-        <x:v>Avery Brooks</x:v>
+        <x:v>Aisha Rahman</x:v>
       </x:c>
       <x:c r="D2" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -687,7 +687,7 @@
         <x:v>72327</x:v>
       </x:c>
       <x:c r="C3" s="16" t="str">
-        <x:v>Jordan Brooks</x:v>
+        <x:v>Mateo Alvarez</x:v>
       </x:c>
       <x:c r="D3" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -707,7 +707,7 @@
         <x:v>83193</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>Taylor Brooks</x:v>
+        <x:v>Priya Shah</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -727,7 +727,7 @@
         <x:v>83194</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>Morgan Brooks</x:v>
+        <x:v>Liam O'Connor</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -747,7 +747,7 @@
         <x:v>83195</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>Riley Brooks</x:v>
+        <x:v>Sofia Rossi</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -767,7 +767,7 @@
         <x:v>83197</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>Casey Brooks</x:v>
+        <x:v>Kenji Sato</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -787,7 +787,7 @@
         <x:v>83199</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
-        <x:v>Quinn Brooks</x:v>
+        <x:v>Mei Chen</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -807,7 +807,7 @@
         <x:v>83200</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
-        <x:v>Parker Brooks</x:v>
+        <x:v>Kwame Mensah</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -827,7 +827,7 @@
         <x:v>83201</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
-        <x:v>Reese Brooks</x:v>
+        <x:v>Fatima Hassan</x:v>
       </x:c>
       <x:c r="D10" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -847,7 +847,7 @@
         <x:v>83202</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
-        <x:v>Cameron Brooks</x:v>
+        <x:v>Noah Williams</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -867,7 +867,7 @@
         <x:v>83203</x:v>
       </x:c>
       <x:c r="C12" s="16" t="str">
-        <x:v>Skyler Brooks</x:v>
+        <x:v>Amara Okafor</x:v>
       </x:c>
       <x:c r="D12" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -887,7 +887,7 @@
         <x:v>83204</x:v>
       </x:c>
       <x:c r="C13" s="16" t="str">
-        <x:v>Rowan Brooks</x:v>
+        <x:v>Diego Morales</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -907,7 +907,7 @@
         <x:v>83205</x:v>
       </x:c>
       <x:c r="C14" s="16" t="str">
-        <x:v>Emerson Brooks</x:v>
+        <x:v>Leila Haddad</x:v>
       </x:c>
       <x:c r="D14" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -927,7 +927,7 @@
         <x:v>83206</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
-        <x:v>Finley Brooks</x:v>
+        <x:v>Arjun Patel</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -947,7 +947,7 @@
         <x:v>83208</x:v>
       </x:c>
       <x:c r="C16" s="16" t="str">
-        <x:v>Dakota Brooks</x:v>
+        <x:v>Hana Kim</x:v>
       </x:c>
       <x:c r="D16" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -967,7 +967,7 @@
         <x:v>83209</x:v>
       </x:c>
       <x:c r="C17" s="16" t="str">
-        <x:v>Hayden Brooks</x:v>
+        <x:v>Lucas Ferreira</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -987,7 +987,7 @@
         <x:v>83210</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
-        <x:v>Sage Brooks</x:v>
+        <x:v>Zara Ali</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1007,7 +1007,7 @@
         <x:v>83212</x:v>
       </x:c>
       <x:c r="C19" s="16" t="str">
-        <x:v>Alex Brooks</x:v>
+        <x:v>Ethan Nguyen</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1027,7 +1027,7 @@
         <x:v>83383</x:v>
       </x:c>
       <x:c r="C20" s="16" t="str">
-        <x:v>Jamie Brooks</x:v>
+        <x:v>Maya Thompson</x:v>
       </x:c>
       <x:c r="D20" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1047,7 +1047,7 @@
         <x:v>83477</x:v>
       </x:c>
       <x:c r="C21" s="16" t="str">
-        <x:v>Kendall Brooks</x:v>
+        <x:v>Samuel Adeyemi</x:v>
       </x:c>
       <x:c r="D21" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1067,7 +1067,7 @@
         <x:v>83478</x:v>
       </x:c>
       <x:c r="C22" s="16" t="str">
-        <x:v>Robin Brooks</x:v>
+        <x:v>Valentina Cruz</x:v>
       </x:c>
       <x:c r="D22" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1087,7 +1087,7 @@
         <x:v>83479</x:v>
       </x:c>
       <x:c r="C23" s="16" t="str">
-        <x:v>Drew Brooks</x:v>
+        <x:v>Omar Khalil</x:v>
       </x:c>
       <x:c r="D23" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1107,7 +1107,7 @@
         <x:v>83480</x:v>
       </x:c>
       <x:c r="C24" s="16" t="str">
-        <x:v>Blair Brooks</x:v>
+        <x:v>Nina Kowalski</x:v>
       </x:c>
       <x:c r="D24" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1127,7 +1127,7 @@
         <x:v>84455</x:v>
       </x:c>
       <x:c r="C25" s="16" t="str">
-        <x:v>Charlie Brooks</x:v>
+        <x:v>Javier Rivera</x:v>
       </x:c>
       <x:c r="D25" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1147,7 +1147,7 @@
         <x:v>85192</x:v>
       </x:c>
       <x:c r="C26" s="16" t="str">
-        <x:v>Lane Brooks</x:v>
+        <x:v>Grace Park</x:v>
       </x:c>
       <x:c r="D26" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1167,7 +1167,7 @@
         <x:v>90216</x:v>
       </x:c>
       <x:c r="C27" s="16" t="str">
-        <x:v>Avery Chen</x:v>
+        <x:v>Malik Johnson</x:v>
       </x:c>
       <x:c r="D27" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1187,7 +1187,7 @@
         <x:v>74864</x:v>
       </x:c>
       <x:c r="C28" s="16" t="str">
-        <x:v>Jordan Chen</x:v>
+        <x:v>Elena Petrova</x:v>
       </x:c>
       <x:c r="D28" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1207,7 +1207,7 @@
         <x:v>79409</x:v>
       </x:c>
       <x:c r="C29" s="16" t="str">
-        <x:v>Taylor Chen</x:v>
+        <x:v>Ravi Desai</x:v>
       </x:c>
       <x:c r="D29" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1227,7 +1227,7 @@
         <x:v>79410</x:v>
       </x:c>
       <x:c r="C30" s="16" t="str">
-        <x:v>Morgan Chen</x:v>
+        <x:v>Camila Santos</x:v>
       </x:c>
       <x:c r="D30" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1247,7 +1247,7 @@
         <x:v>79411</x:v>
       </x:c>
       <x:c r="C31" s="16" t="str">
-        <x:v>Riley Chen</x:v>
+        <x:v>Yusuf Ahmed</x:v>
       </x:c>
       <x:c r="D31" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1267,7 +1267,7 @@
         <x:v>79412</x:v>
       </x:c>
       <x:c r="C32" s="16" t="str">
-        <x:v>Casey Chen</x:v>
+        <x:v>Isabella Romano</x:v>
       </x:c>
       <x:c r="D32" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1287,7 +1287,7 @@
         <x:v>79413</x:v>
       </x:c>
       <x:c r="C33" s="16" t="str">
-        <x:v>Quinn Chen</x:v>
+        <x:v>Daniel Cho</x:v>
       </x:c>
       <x:c r="D33" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1307,7 +1307,7 @@
         <x:v>79414</x:v>
       </x:c>
       <x:c r="C34" s="16" t="str">
-        <x:v>Parker Chen</x:v>
+        <x:v>Nadia Ibrahim</x:v>
       </x:c>
       <x:c r="D34" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1327,7 +1327,7 @@
         <x:v>79415</x:v>
       </x:c>
       <x:c r="C35" s="16" t="str">
-        <x:v>Reese Chen</x:v>
+        <x:v>Andre Baptiste</x:v>
       </x:c>
       <x:c r="D35" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1347,7 +1347,7 @@
         <x:v>79416</x:v>
       </x:c>
       <x:c r="C36" s="16" t="str">
-        <x:v>Cameron Chen</x:v>
+        <x:v>Sienna Martin</x:v>
       </x:c>
       <x:c r="D36" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1367,7 +1367,7 @@
         <x:v>79417</x:v>
       </x:c>
       <x:c r="C37" s="16" t="str">
-        <x:v>Skyler Chen</x:v>
+        <x:v>Marcus Brown</x:v>
       </x:c>
       <x:c r="D37" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1387,7 +1387,7 @@
         <x:v>79419</x:v>
       </x:c>
       <x:c r="C38" s="16" t="str">
-        <x:v>Rowan Chen</x:v>
+        <x:v>Ana Popescu</x:v>
       </x:c>
       <x:c r="D38" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1407,7 +1407,7 @@
         <x:v>79420</x:v>
       </x:c>
       <x:c r="C39" s="16" t="str">
-        <x:v>Emerson Chen</x:v>
+        <x:v>Tariq Mahmoud</x:v>
       </x:c>
       <x:c r="D39" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1427,7 +1427,7 @@
         <x:v>79577</x:v>
       </x:c>
       <x:c r="C40" s="16" t="str">
-        <x:v>Finley Chen</x:v>
+        <x:v>Lucia Garcia</x:v>
       </x:c>
       <x:c r="D40" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1447,7 +1447,7 @@
         <x:v>79578</x:v>
       </x:c>
       <x:c r="C41" s="16" t="str">
-        <x:v>Dakota Chen</x:v>
+        <x:v>Jonah Stein</x:v>
       </x:c>
       <x:c r="D41" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1467,7 +1467,7 @@
         <x:v>79579</x:v>
       </x:c>
       <x:c r="C42" s="16" t="str">
-        <x:v>Hayden Chen</x:v>
+        <x:v>Imani Carter</x:v>
       </x:c>
       <x:c r="D42" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1487,7 +1487,7 @@
         <x:v>79580</x:v>
       </x:c>
       <x:c r="C43" s="16" t="str">
-        <x:v>Sage Chen</x:v>
+        <x:v>Theo Laurent</x:v>
       </x:c>
       <x:c r="D43" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1507,7 +1507,7 @@
         <x:v>79581</x:v>
       </x:c>
       <x:c r="C44" s="16" t="str">
-        <x:v>Alex Chen</x:v>
+        <x:v>Mina Yamamoto</x:v>
       </x:c>
       <x:c r="D44" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1527,7 +1527,7 @@
         <x:v>79582</x:v>
       </x:c>
       <x:c r="C45" s="16" t="str">
-        <x:v>Jamie Chen</x:v>
+        <x:v>Alejandro Torres</x:v>
       </x:c>
       <x:c r="D45" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1547,7 +1547,7 @@
         <x:v>79583</x:v>
       </x:c>
       <x:c r="C46" s="16" t="str">
-        <x:v>Kendall Chen</x:v>
+        <x:v>Chloe Dubois</x:v>
       </x:c>
       <x:c r="D46" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1567,7 +1567,7 @@
         <x:v>79584</x:v>
       </x:c>
       <x:c r="C47" s="16" t="str">
-        <x:v>Robin Chen</x:v>
+        <x:v>Bilal Khan</x:v>
       </x:c>
       <x:c r="D47" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1587,7 +1587,7 @@
         <x:v>79585</x:v>
       </x:c>
       <x:c r="C48" s="16" t="str">
-        <x:v>Drew Chen</x:v>
+        <x:v>Ava Sinclair</x:v>
       </x:c>
       <x:c r="D48" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1607,7 +1607,7 @@
         <x:v>79586</x:v>
       </x:c>
       <x:c r="C49" s="16" t="str">
-        <x:v>Blair Chen</x:v>
+        <x:v>Kofi Boateng</x:v>
       </x:c>
       <x:c r="D49" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1627,7 +1627,7 @@
         <x:v>79587</x:v>
       </x:c>
       <x:c r="C50" s="16" t="str">
-        <x:v>Charlie Chen</x:v>
+        <x:v>Layla Mansour</x:v>
       </x:c>
       <x:c r="D50" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1647,7 +1647,7 @@
         <x:v>79588</x:v>
       </x:c>
       <x:c r="C51" s="16" t="str">
-        <x:v>Lane Chen</x:v>
+        <x:v>Gabriel Silva</x:v>
       </x:c>
       <x:c r="D51" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1667,7 +1667,7 @@
         <x:v>79589</x:v>
       </x:c>
       <x:c r="C52" s="16" t="str">
-        <x:v>Avery Davis</x:v>
+        <x:v>Neha Kapoor</x:v>
       </x:c>
       <x:c r="D52" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1687,7 +1687,7 @@
         <x:v>80906</x:v>
       </x:c>
       <x:c r="C53" s="16" t="str">
-        <x:v>Jordan Davis</x:v>
+        <x:v>Milan Jovanovic</x:v>
       </x:c>
       <x:c r="D53" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1707,7 +1707,7 @@
         <x:v>83960</x:v>
       </x:c>
       <x:c r="C54" s="16" t="str">
-        <x:v>Taylor Davis</x:v>
+        <x:v>Rosa Martinez</x:v>
       </x:c>
       <x:c r="D54" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1727,7 +1727,7 @@
         <x:v>83967</x:v>
       </x:c>
       <x:c r="C55" s="16" t="str">
-        <x:v>Morgan Davis</x:v>
+        <x:v>Isaac Cohen</x:v>
       </x:c>
       <x:c r="D55" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1747,7 +1747,7 @@
         <x:v>84823</x:v>
       </x:c>
       <x:c r="C56" s="16" t="str">
-        <x:v>Riley Davis</x:v>
+        <x:v>Adanna Eze</x:v>
       </x:c>
       <x:c r="D56" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1767,7 +1767,7 @@
         <x:v>84826</x:v>
       </x:c>
       <x:c r="C57" s="16" t="str">
-        <x:v>Casey Davis</x:v>
+        <x:v>Hugo Moreau</x:v>
       </x:c>
       <x:c r="D57" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1787,7 +1787,7 @@
         <x:v>84828</x:v>
       </x:c>
       <x:c r="C58" s="16" t="str">
-        <x:v>Quinn Davis</x:v>
+        <x:v>Salma Nasser</x:v>
       </x:c>
       <x:c r="D58" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1807,7 +1807,7 @@
         <x:v>84834</x:v>
       </x:c>
       <x:c r="C59" s="16" t="str">
-        <x:v>Parker Davis</x:v>
+        <x:v>Benjamin Lee</x:v>
       </x:c>
       <x:c r="D59" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1827,7 +1827,7 @@
         <x:v>84835</x:v>
       </x:c>
       <x:c r="C60" s="16" t="str">
-        <x:v>Reese Davis</x:v>
+        <x:v>Freya Andersen</x:v>
       </x:c>
       <x:c r="D60" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1847,7 +1847,7 @@
         <x:v>84836</x:v>
       </x:c>
       <x:c r="C61" s="16" t="str">
-        <x:v>Cameron Davis</x:v>
+        <x:v>Nikhil Rao</x:v>
       </x:c>
       <x:c r="D61" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1867,7 +1867,7 @@
         <x:v>84837</x:v>
       </x:c>
       <x:c r="C62" s="16" t="str">
-        <x:v>Skyler Davis</x:v>
+        <x:v>Keira Murphy</x:v>
       </x:c>
       <x:c r="D62" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1887,7 +1887,7 @@
         <x:v>84838</x:v>
       </x:c>
       <x:c r="C63" s="16" t="str">
-        <x:v>Rowan Davis</x:v>
+        <x:v>Darius Walker</x:v>
       </x:c>
       <x:c r="D63" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1907,7 +1907,7 @@
         <x:v>87863</x:v>
       </x:c>
       <x:c r="C64" s="16" t="str">
-        <x:v>Emerson Davis</x:v>
+        <x:v>Yuna Tanaka</x:v>
       </x:c>
       <x:c r="D64" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1927,7 +1927,7 @@
         <x:v>87864</x:v>
       </x:c>
       <x:c r="C65" s="16" t="str">
-        <x:v>Finley Davis</x:v>
+        <x:v>Pedro Castillo</x:v>
       </x:c>
       <x:c r="D65" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1947,7 +1947,7 @@
         <x:v>87865</x:v>
       </x:c>
       <x:c r="C66" s="16" t="str">
-        <x:v>Dakota Davis</x:v>
+        <x:v>Maryam Farouk</x:v>
       </x:c>
       <x:c r="D66" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1967,7 +1967,7 @@
         <x:v>87866</x:v>
       </x:c>
       <x:c r="C67" s="16" t="str">
-        <x:v>Hayden Davis</x:v>
+        <x:v>Sebastian Mueller</x:v>
       </x:c>
       <x:c r="D67" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -1987,7 +1987,7 @@
         <x:v>87867</x:v>
       </x:c>
       <x:c r="C68" s="16" t="str">
-        <x:v>Sage Davis</x:v>
+        <x:v>Ayana Robinson</x:v>
       </x:c>
       <x:c r="D68" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2007,7 +2007,7 @@
         <x:v>87868</x:v>
       </x:c>
       <x:c r="C69" s="16" t="str">
-        <x:v>Alex Davis</x:v>
+        <x:v>Vikram Mehta</x:v>
       </x:c>
       <x:c r="D69" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2027,7 +2027,7 @@
         <x:v>87869</x:v>
       </x:c>
       <x:c r="C70" s="16" t="str">
-        <x:v>Jamie Davis</x:v>
+        <x:v>Clara Jensen</x:v>
       </x:c>
       <x:c r="D70" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2047,7 +2047,7 @@
         <x:v>87870</x:v>
       </x:c>
       <x:c r="C71" s="16" t="str">
-        <x:v>Kendall Davis</x:v>
+        <x:v>Jamal Wilson</x:v>
       </x:c>
       <x:c r="D71" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2067,7 +2067,7 @@
         <x:v>87871</x:v>
       </x:c>
       <x:c r="C72" s="16" t="str">
-        <x:v>Robin Davis</x:v>
+        <x:v>Iris Zhang</x:v>
       </x:c>
       <x:c r="D72" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2087,7 +2087,7 @@
         <x:v>87873</x:v>
       </x:c>
       <x:c r="C73" s="16" t="str">
-        <x:v>Drew Davis</x:v>
+        <x:v>Dominic Russo</x:v>
       </x:c>
       <x:c r="D73" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2107,7 +2107,7 @@
         <x:v>87874</x:v>
       </x:c>
       <x:c r="C74" s="16" t="str">
-        <x:v>Blair Davis</x:v>
+        <x:v>Lina Saad</x:v>
       </x:c>
       <x:c r="D74" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2127,7 +2127,7 @@
         <x:v>87875</x:v>
       </x:c>
       <x:c r="C75" s="16" t="str">
-        <x:v>Charlie Davis</x:v>
+        <x:v>Xavier Morgan</x:v>
       </x:c>
       <x:c r="D75" s="16" t="str">
         <x:v>TRUE</x:v>
@@ -2147,7 +2147,7 @@
         <x:v>87876</x:v>
       </x:c>
       <x:c r="C76" s="30" t="str">
-        <x:v>Lane Davis</x:v>
+        <x:v>Amina Diallo</x:v>
       </x:c>
       <x:c r="D76" s="30" t="str">
         <x:v>TRUE</x:v>
@@ -2167,7 +2167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R031189601f144051"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra559f49edccb4ee6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>